<commit_message>
Add deal access control feature with private visibility checks
</commit_message>
<xml_diff>
--- a/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
+++ b/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyProjects\Capgemini_Sprint\FreeCRMQualityAssurance\Automation_Testing\selenium-ui-automation\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE82E030-5F72-4322-99E5-64C3D00112A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB9B1F-3638-4809-A279-1B907A600B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Deals" sheetId="1" r:id="rId1"/>
+    <sheet name="Credentials" sheetId="2" r:id="rId1"/>
+    <sheet name="Deals" sheetId="1" r:id="rId2"/>
+    <sheet name="Tasks" sheetId="3" r:id="rId3"/>
+    <sheet name="Contacts" sheetId="4" r:id="rId4"/>
+    <sheet name="Company" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
   <si>
     <t>Title</t>
   </si>
@@ -67,16 +71,183 @@
   </si>
   <si>
     <t>Probablity</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>pathaksudeshna92@gmail.com</t>
+  </si>
+  <si>
+    <t>Sudeshna@Crm1</t>
+  </si>
+  <si>
+    <t>snehashism93@gmail.com</t>
+  </si>
+  <si>
+    <t>Iem@2026</t>
+  </si>
+  <si>
+    <t>subhangip2005@outlook.com</t>
+  </si>
+  <si>
+    <t>snehalghosh22@gmail.com</t>
+  </si>
+  <si>
+    <t>Access Control Test Deal</t>
+  </si>
+  <si>
+    <t>userName</t>
+  </si>
+  <si>
+    <t>Snehashis Mandel</t>
+  </si>
+  <si>
+    <t>Subhangi Pandey</t>
+  </si>
+  <si>
+    <t>Snehal Ghosh</t>
+  </si>
+  <si>
+    <t>Due Data</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Debashis</t>
+  </si>
+  <si>
+    <t>Mandal</t>
+  </si>
+  <si>
+    <t>mandaldebashis62@gmail.com</t>
+  </si>
+  <si>
+    <t>Phone Country Code</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Phone Type</t>
+  </si>
+  <si>
+    <t>Email Type</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Social site</t>
+  </si>
+  <si>
+    <t>Social ID</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
+    <t>Num. of Employees</t>
+  </si>
+  <si>
+    <t>Annual Revenue</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>VAT Number</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>+91</t>
+  </si>
+  <si>
+    <t>80 4444 9876</t>
+  </si>
+  <si>
+    <t>Work</t>
+  </si>
+  <si>
+    <t>partnerships@bluehorizon.com</t>
+  </si>
+  <si>
+    <t>A regional IT consultancy that bundles our cloud storage products with their hardware sales</t>
+  </si>
+  <si>
+    <t>Twitter</t>
+  </si>
+  <si>
+    <t>@BlueHorizonIT</t>
+  </si>
+  <si>
+    <t>Information Technology</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>Partner</t>
+  </si>
+  <si>
+    <t>GSTIN9876543210A2</t>
+  </si>
+  <si>
+    <t>PART-505</t>
+  </si>
+  <si>
+    <t>Quantum FinTech Solutions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -99,14 +270,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -418,10 +596,92 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8898A123-6092-4ECE-BE39-05E0984528A3}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD7A47D-9843-4061-A122-3A2B8DE4D055}">
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{015DF69F-016D-4B87-91B8-733480D91E3E}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{267761C4-778F-492B-9D65-0D0EDF0EA3CA}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{C581BDDA-E1B8-4282-860E-7298EF6292CD}"/>
+    <hyperlink ref="A4" r:id="rId4" xr:uid="{10CECF2A-CA2F-4D8D-8310-9E4AD3C55A47}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{B9A87C6A-0D65-4077-AF8B-F160ECA13E2F}"/>
+    <hyperlink ref="B5" r:id="rId6" xr:uid="{06D3BB99-528A-4D42-BA6C-C2AAF4B33F37}"/>
+    <hyperlink ref="B3" r:id="rId7" xr:uid="{4732D7BA-4E48-4C2E-AEE4-BDFE3D55C086}"/>
+    <hyperlink ref="A5" r:id="rId8" xr:uid="{B6DB9077-4EB4-450F-865F-C19B8265B26E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8898A123-6092-4ECE-BE39-05E0984528A3}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -472,27 +732,240 @@
         <v>46129</v>
       </c>
     </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <v>5000</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>80</v>
+      </c>
+      <c r="G3" s="1">
+        <v>46130</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018B913E-E9EF-4854-9328-AC3CF717FA43}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="3">
+        <v>46137</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387EB7D3-DA84-4B00-8743-BB4AF6C4141D}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{65428618-F916-40F7-B3B4-4DB01FFF1775}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE21098C-135E-4080-8BAB-4EE6885FFB51}">
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="76.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" s="5">
+        <v>150</v>
+      </c>
+      <c r="K2" s="5">
+        <v>85000000</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F055B28FFEB2A0418F25EB5BF07F1E83" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d0f07cab075b6f743d602f5367b62e3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7271d819-4382-409a-9171-0e558f844953" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f725e4be6f41bd12717ee6588a206a97" ns3:_="">
     <xsd:import namespace="7271d819-4382-409a-9171-0e558f844953"/>
@@ -668,31 +1141,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7271d819-4382-409a-9171-0e558f844953"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4AC84AA-F2C4-4320-AD32-5E17AAE25130}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -708,4 +1172,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7271d819-4382-409a-9171-0e558f844953"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update delete contact step and feature tags for consistency
</commit_message>
<xml_diff>
--- a/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
+++ b/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SUBHANGI\Desktop\FreeCRMQualityAssurance\Automation_Testing\selenium-ui-automation\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyProjects\Capgemini_Sprint\FreeCRMQualityAssurance\Automation_Testing\selenium-ui-automation\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644E012C-94E6-4996-A3AA-A1B93FDED56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB9B1F-3638-4809-A279-1B907A600B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Credentials" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
   <si>
     <t>Title</t>
   </si>
@@ -112,6 +112,9 @@
     <t>Snehal Ghosh</t>
   </si>
   <si>
+    <t>Due Data</t>
+  </si>
+  <si>
     <t>Task</t>
   </si>
   <si>
@@ -221,22 +224,13 @@
   </si>
   <si>
     <t>Quantum FinTech Solutions</t>
-  </si>
-  <si>
-    <t>25-04-2026  00:00:00</t>
-  </si>
-  <si>
-    <t>Due Date</t>
-  </si>
-  <si>
-    <t>Reviewing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,10 +251,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9.8000000000000007"/>
-      <name val="JetBrains Mono"/>
     </font>
   </fonts>
   <fills count="2">
@@ -284,14 +274,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -311,9 +301,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -351,7 +341,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -457,7 +447,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -599,7 +589,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -608,14 +598,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD7A47D-9843-4061-A122-3A2B8DE4D055}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -626,7 +616,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -637,7 +627,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -648,7 +638,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -659,7 +649,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -689,14 +679,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8898A123-6092-4ECE-BE39-05E0984528A3}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -719,7 +709,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -742,7 +732,7 @@
         <v>46129</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -772,78 +762,63 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018B913E-E9EF-4854-9328-AC3CF717FA43}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" t="s">
-        <v>63</v>
+        <v>25</v>
+      </c>
+      <c r="B2" s="3">
+        <v>46137</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387EB7D3-DA84-4B00-8743-BB4AF6C4141D}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="C1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>30</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -856,8 +831,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE21098C-135E-4080-8BAB-4EE6885FFB51}">
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
@@ -869,117 +844,121 @@
     <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
-      <c r="A1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="C1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F1" t="s">
+      <c r="D1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G1" t="s">
+      <c r="F1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H1" t="s">
+      <c r="G1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="I1" t="s">
+      <c r="H1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J1" t="s">
+      <c r="I1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="K1" t="s">
+      <c r="J1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="L1" t="s">
+      <c r="K1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="M1" t="s">
+      <c r="L1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="N1" t="s">
-        <v>42</v>
-      </c>
-      <c r="O1" t="s">
+      <c r="N1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="P1" t="s">
+      <c r="O1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="P1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="R1" t="s">
+      <c r="Q1" s="5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="A2" s="3" t="s">
+      <c r="R1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B2" t="s">
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G2" t="s">
+      <c r="E2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H2" t="s">
+      <c r="G2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J2">
+      <c r="I2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" s="5">
         <v>150</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="5">
         <v>85000000</v>
       </c>
-      <c r="L2" t="s">
-        <v>55</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="L2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N2" t="s">
-        <v>56</v>
-      </c>
-      <c r="O2" t="s">
+      <c r="N2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="P2" t="s">
+      <c r="O2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="P2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="R2" t="s">
+      <c r="Q2" s="5" t="s">
         <v>60</v>
       </c>
+      <c r="R2" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -987,21 +966,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F055B28FFEB2A0418F25EB5BF07F1E83" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d0f07cab075b6f743d602f5367b62e3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7271d819-4382-409a-9171-0e558f844953" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f725e4be6f41bd12717ee6588a206a97" ns3:_="">
     <xsd:import namespace="7271d819-4382-409a-9171-0e558f844953"/>
@@ -1177,31 +1141,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7271d819-4382-409a-9171-0e558f844953"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4AC84AA-F2C4-4320-AD32-5E17AAE25130}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1217,4 +1172,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7271d819-4382-409a-9171-0e558f844953"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Cleaning Apache POI changes
</commit_message>
<xml_diff>
--- a/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
+++ b/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyProjects\Capgemini_Sprint\FreeCRMQualityAssurance\Automation_Testing\selenium-ui-automation\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SUBHANGI\Desktop\FreeCRMQualityAssurance\Automation_Testing\selenium-ui-automation\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB9B1F-3638-4809-A279-1B907A600B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644E012C-94E6-4996-A3AA-A1B93FDED56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Credentials" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="64">
   <si>
     <t>Title</t>
   </si>
@@ -112,9 +112,6 @@
     <t>Snehal Ghosh</t>
   </si>
   <si>
-    <t>Due Data</t>
-  </si>
-  <si>
     <t>Task</t>
   </si>
   <si>
@@ -224,13 +221,22 @@
   </si>
   <si>
     <t>Quantum FinTech Solutions</t>
+  </si>
+  <si>
+    <t>25-04-2026  00:00:00</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Reviewing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,6 +257,10 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <name val="JetBrains Mono"/>
     </font>
   </fonts>
   <fills count="2">
@@ -274,14 +284,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -301,9 +311,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -341,7 +351,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -447,7 +457,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -589,7 +599,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -598,14 +608,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD7A47D-9843-4061-A122-3A2B8DE4D055}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="26.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -616,7 +626,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -627,7 +637,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -638,7 +648,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -649,7 +659,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -679,14 +689,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8898A123-6092-4ECE-BE39-05E0984528A3}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -709,7 +719,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -732,7 +742,7 @@
         <v>46129</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -762,63 +772,78 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018B913E-E9EF-4854-9328-AC3CF717FA43}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="3">
-        <v>46137</v>
+      <c r="B2" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387EB7D3-DA84-4B00-8743-BB4AF6C4141D}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="5" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -831,8 +856,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE21098C-135E-4080-8BAB-4EE6885FFB51}">
-  <dimension ref="A1:T2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
@@ -844,121 +869,117 @@
     <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:18">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" t="s">
         <v>43</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" t="s">
         <v>44</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="5" t="s">
+    </row>
+    <row r="2" spans="1:18">
+      <c r="A2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B2" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2">
+        <v>150</v>
+      </c>
+      <c r="K2">
+        <v>85000000</v>
+      </c>
+      <c r="L2" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="5">
-        <v>150</v>
-      </c>
-      <c r="K2" s="5">
-        <v>85000000</v>
-      </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" t="s">
         <v>56</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" t="s">
         <v>57</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" t="s">
         <v>58</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" t="s">
         <v>59</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" t="s">
         <v>60</v>
       </c>
-      <c r="R2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -966,6 +987,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F055B28FFEB2A0418F25EB5BF07F1E83" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d0f07cab075b6f743d602f5367b62e3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7271d819-4382-409a-9171-0e558f844953" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f725e4be6f41bd12717ee6588a206a97" ns3:_="">
     <xsd:import namespace="7271d819-4382-409a-9171-0e558f844953"/>
@@ -1141,22 +1177,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7271d819-4382-409a-9171-0e558f844953"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4AC84AA-F2C4-4320-AD32-5E17AAE25130}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1172,28 +1217,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7271d819-4382-409a-9171-0e558f844953"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Excel to final Version
</commit_message>
<xml_diff>
--- a/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
+++ b/Automation_Testing/selenium-ui-automation/src/test/resources/testData/FreeCRM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyProjects\Capgemini_Sprint\FreeCRMQualityAssurance\Automation_Testing\selenium-ui-automation\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB9B1F-3638-4809-A279-1B907A600B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98FBCE1F-FA86-4CF9-AADA-0A97309EF179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8B8F7499-8A40-46D9-9F65-A4F238397EF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Credentials" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
   <si>
     <t>Title</t>
   </si>
@@ -112,9 +112,6 @@
     <t>Snehal Ghosh</t>
   </si>
   <si>
-    <t>Due Data</t>
-  </si>
-  <si>
     <t>Task</t>
   </si>
   <si>
@@ -224,6 +221,30 @@
   </si>
   <si>
     <t>Quantum FinTech Solutions</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>Nvidia GPU</t>
+  </si>
+  <si>
+    <t>Meeting with client</t>
+  </si>
+  <si>
+    <t>Vikram Singh</t>
+  </si>
+  <si>
+    <t>Follow up</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Reviewing</t>
   </si>
 </sst>
 </file>
@@ -274,14 +295,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -678,15 +697,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8898A123-6092-4ECE-BE39-05E0984528A3}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -708,8 +732,23 @@
       <c r="G1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -723,7 +762,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F2">
         <v>75</v>
@@ -731,8 +770,23 @@
       <c r="G2" s="1">
         <v>46129</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K2" t="s">
+        <v>64</v>
+      </c>
+      <c r="L2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -762,26 +816,39 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018B913E-E9EF-4854-9328-AC3CF717FA43}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="3">
+      <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1">
         <v>46137</v>
+      </c>
+      <c r="D2" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -800,25 +867,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="5" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -831,7 +898,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE21098C-135E-4080-8BAB-4EE6885FFB51}">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -844,121 +911,117 @@
     <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" t="s">
         <v>43</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" t="s">
         <v>44</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="5" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B2" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2">
+        <v>150</v>
+      </c>
+      <c r="K2">
+        <v>85000000</v>
+      </c>
+      <c r="L2" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="5">
-        <v>150</v>
-      </c>
-      <c r="K2" s="5">
-        <v>85000000</v>
-      </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" t="s">
         <v>56</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" t="s">
         <v>57</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" t="s">
         <v>58</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" t="s">
         <v>59</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" t="s">
         <v>60</v>
       </c>
-      <c r="R2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1142,18 +1205,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1175,14 +1238,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7994A2-6E55-4585-85D4-227A6677CDA5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -1196,4 +1251,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46C4BA0C-9E43-4FEF-9DF9-4D06CBD4BC3D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>